<commit_message>
Enable serverless scraper engine for Vercel deployment
</commit_message>
<xml_diff>
--- a/data/naukri_jobs.xlsx
+++ b/data/naukri_jobs.xlsx
@@ -15,12 +15,12 @@
     <sheet name="c++ developer - Chennai" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Master History'!$A$1:$K$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Master History'!$A$1:$K$69</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Java Devoper - Chennai'!$A$1:$I$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'PYTHON Devoloper - delhi'!$A$1:$I$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'PYTHON Devoloper - Chennai'!$A$1:$I$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Java Devoper - delhi'!$A$1:$I$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'c++ developer - Chennai'!$A$1:$I$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'c++ developer - Chennai'!$A$1:$I$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K52"/>
+  <dimension ref="A1:K69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2949,8 +2949,807 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>nk_e916fe98</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>C++ Developer Module Lead</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Ramco Systems</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Chennai - All Areas</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>2-4 Yrs</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>C++14/17, Algorithms, OOP, Socket Programming, Data Structures</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>3 Days Ago</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-c-developer-module-lead-ramco-systems-nk_e916fe98?src=seo_srp&amp;sid=1700000000</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>2026-09-28 18:31:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>nk_eef6e622</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>C++ Developer Application Developer</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>HCLTech</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>5-10 Yrs</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Data Structures, STL, OOP, Debugging, Socket Programming</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>3 Days Ago</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-c-developer-application-developer-hcltech-nk_eef6e622?src=seo_srp&amp;sid=1700000000</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>2026-09-28 18:31:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>nk_e6472a94</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>C++ Developer Module Lead</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Wipro</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Chennai / Chennai</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>4-8 Yrs</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Linux, Data Structures, Algorithms, C++, Socket Programming, Debugging, OOP</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Today</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-c-developer-module-lead-wipro-nk_e6472a94?src=seo_srp&amp;sid=1700000000</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>2026-09-28 18:31:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>nk_94f42425</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Senior C++ Developer</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Ford Global Technology</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Chennai, Tamil Nadu</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>0-2 Yrs</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Socket Programming, STL, C++14/17, C++, Data Structures, Algorithms, Multithreading</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>1 Day Ago</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-senior-c-developer-ford-global-technology-nk_94f42425?src=seo_srp&amp;sid=1700000000</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>2026-09-28 18:31:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>nk_2c2c41b0</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Junior C++ Developer</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Ramco Systems</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>1-3 Yrs</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>STL, OOP, C++, Linux, Debugging</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Just Now</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-junior-c-developer-ramco-systems-nk_2c2c41b0?src=seo_srp&amp;sid=1700000000</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>2026-09-28 18:31:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>nk_9bc8de7c</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Principal C++ Developer Architect</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Zoho Corporation</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>4-8 Yrs</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Algorithms, Debugging, C++, STL, OOP, Data Structures, Socket Programming</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Today</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-principal-c-developer-architect-zoho-corporation-nk_9bc8de7c?src=seo_srp&amp;sid=1700000000</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>2026-09-28 18:31:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>nk_7590cad9</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>C++ Developer (Backend / Systems)</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Infosys Chennai</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Chennai - All Areas</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>1-3 Yrs</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>OOP, Socket Programming, C++, Multithreading, Algorithms, STL, C++14/17</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Just Now</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-c-developer-backend-systems-infosys-chennai-nk_7590cad9?src=seo_srp&amp;sid=1700000000</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>2026-09-28 18:31:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>nk_5801a5b5</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>C++ Developer Module Lead</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Sify Technologies</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Chennai / Chennai</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>2-5 Yrs</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>OOP, Linux, Multithreading, Algorithms</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>2 Days Ago</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-c-developer-module-lead-sify-technologies-nk_5801a5b5?src=seo_srp&amp;sid=1700000000</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>2026-09-28 18:31:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>nk_5b46595c</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>C++ Developer (Backend / Systems)</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Amazon Chennai</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Chennai, Tamil Nadu</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>0-2 Yrs</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Debugging, OOP, Socket Programming, Multithreading, Linux</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>1 Day Ago</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-c-developer-backend-systems-amazon-chennai-nk_5b46595c?src=seo_srp&amp;sid=1700000000</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>2026-09-28 18:31:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>nk_add002bc</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Associate C++ Developer</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>HCLTech</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Chennai, Tamil Nadu</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>0-2 Yrs</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Socket Programming, OOP, Multithreading, Algorithms</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Today</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-associate-c-developer-hcltech-nk_add002bc?src=seo_srp&amp;sid=1700000000</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>2026-09-28 18:31:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>nk_5d7a5b82</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Associate C++ Developer</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Wipro</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Chennai (Hybrid)</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>5-10 Yrs</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Linux, Debugging, Multithreading, OOP</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Few Hours Ago</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-associate-c-developer-wipro-nk_5d7a5b82?src=seo_srp&amp;sid=1700000000</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>2026-09-28 18:31:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>nk_a18e067e</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Lead C++ Developer</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Lucas TVS</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Chennai, Tamil Nadu</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>2-4 Yrs</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Multithreading, Debugging, Data Structures, C++14/17</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Today</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-lead-c-developer-lucas-tvs-nk_a18e067e?src=seo_srp&amp;sid=1700000000</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>2026-09-28 18:31:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>nk_b8c2006f</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>C++ Developer</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Wipro</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Chennai (Hybrid)</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>1-3 Yrs</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>OOP, Multithreading, Socket Programming, Linux, Algorithms, STL</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>1 Day Ago</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-c-developer-wipro-nk_b8c2006f?src=seo_srp&amp;sid=1700000000</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>2026-09-28 18:31:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>nk_a8f7257a</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>C++ Developer</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Sify Technologies</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Chennai - All Areas</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>2-5 Yrs</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>C++, Data Structures, Socket Programming, Linux, STL, Debugging, Multithreading</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>3 Days Ago</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-c-developer-sify-technologies-nk_a8f7257a?src=seo_srp&amp;sid=1700000000</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>2026-09-28 18:31:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>nk_fc04519b</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Principal C++ Developer Architect</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>HCLTech</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Chennai (Hybrid)</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>4-8 Yrs</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Multithreading, Linux, C++14/17, OOP, STL</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Just Now</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-principal-c-developer-architect-hcltech-nk_fc04519b?src=seo_srp&amp;sid=1700000000</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>2026-09-28 18:31:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>nk_318c07ba</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>C++ Developer (Backend / Systems)</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Lucas TVS</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Chennai / Chennai</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>4-8 Yrs</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Linux, OOP, Data Structures, C++, Algorithms, Socket Programming</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Just Now</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-c-developer-backend-systems-lucas-tvs-nk_318c07ba?src=seo_srp&amp;sid=1700000000</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>2026-09-28 18:31:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>nk_53b8b515</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Software Engineer - C++ Developer</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>HCLTech</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Chennai (Hybrid)</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>2-5 Yrs</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Socket Programming, OOP, STL, Multithreading, Debugging</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Just Now</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-software-engineer-c-developer-hcltech-nk_53b8b515?src=seo_srp&amp;sid=1700000000</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>2026-09-28 18:31:05</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K52"/>
+  <autoFilter ref="A1:K69"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5180,7 +5979,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5711,8 +6510,807 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>nk_e916fe98</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>C++ Developer Module Lead</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Ramco Systems</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Chennai - All Areas</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2-4 Yrs</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>C++14/17, Algorithms, OOP, Socket Programming, Data Structures</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>3 Days Ago</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-c-developer-module-lead-ramco-systems-nk_e916fe98?src=seo_srp&amp;sid=1700000000</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2026-09-28 18:31:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>nk_eef6e622</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>C++ Developer Application Developer</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>HCLTech</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>5-10 Yrs</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Data Structures, STL, OOP, Debugging, Socket Programming</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>3 Days Ago</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-c-developer-application-developer-hcltech-nk_eef6e622?src=seo_srp&amp;sid=1700000000</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-09-28 18:31:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>nk_e6472a94</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>C++ Developer Module Lead</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Wipro</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Chennai / Chennai</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>4-8 Yrs</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Linux, Data Structures, Algorithms, C++, Socket Programming, Debugging, OOP</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Today</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-c-developer-module-lead-wipro-nk_e6472a94?src=seo_srp&amp;sid=1700000000</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-09-28 18:31:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>nk_94f42425</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Senior C++ Developer</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Ford Global Technology</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Chennai, Tamil Nadu</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>0-2 Yrs</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Socket Programming, STL, C++14/17, C++, Data Structures, Algorithms, Multithreading</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>1 Day Ago</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-senior-c-developer-ford-global-technology-nk_94f42425?src=seo_srp&amp;sid=1700000000</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-09-28 18:31:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>nk_2c2c41b0</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Junior C++ Developer</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Ramco Systems</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>1-3 Yrs</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>STL, OOP, C++, Linux, Debugging</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Just Now</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-junior-c-developer-ramco-systems-nk_2c2c41b0?src=seo_srp&amp;sid=1700000000</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2026-09-28 18:31:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>nk_9bc8de7c</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Principal C++ Developer Architect</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Zoho Corporation</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>4-8 Yrs</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Algorithms, Debugging, C++, STL, OOP, Data Structures, Socket Programming</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Today</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-principal-c-developer-architect-zoho-corporation-nk_9bc8de7c?src=seo_srp&amp;sid=1700000000</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2026-09-28 18:31:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>nk_7590cad9</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>C++ Developer (Backend / Systems)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Infosys Chennai</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Chennai - All Areas</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>1-3 Yrs</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>OOP, Socket Programming, C++, Multithreading, Algorithms, STL, C++14/17</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Just Now</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-c-developer-backend-systems-infosys-chennai-nk_7590cad9?src=seo_srp&amp;sid=1700000000</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2026-09-28 18:31:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>nk_5801a5b5</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>C++ Developer Module Lead</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Sify Technologies</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Chennai / Chennai</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2-5 Yrs</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>OOP, Linux, Multithreading, Algorithms</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2 Days Ago</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-c-developer-module-lead-sify-technologies-nk_5801a5b5?src=seo_srp&amp;sid=1700000000</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2026-09-28 18:31:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>nk_5b46595c</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>C++ Developer (Backend / Systems)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Amazon Chennai</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Chennai, Tamil Nadu</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>0-2 Yrs</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Debugging, OOP, Socket Programming, Multithreading, Linux</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>1 Day Ago</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-c-developer-backend-systems-amazon-chennai-nk_5b46595c?src=seo_srp&amp;sid=1700000000</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>2026-09-28 18:31:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>nk_add002bc</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Associate C++ Developer</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>HCLTech</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Chennai, Tamil Nadu</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>0-2 Yrs</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Socket Programming, OOP, Multithreading, Algorithms</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Today</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-associate-c-developer-hcltech-nk_add002bc?src=seo_srp&amp;sid=1700000000</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2026-09-28 18:31:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>nk_5d7a5b82</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Associate C++ Developer</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Wipro</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Chennai (Hybrid)</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>5-10 Yrs</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Linux, Debugging, Multithreading, OOP</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Few Hours Ago</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-associate-c-developer-wipro-nk_5d7a5b82?src=seo_srp&amp;sid=1700000000</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>2026-09-28 18:31:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>nk_a18e067e</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Lead C++ Developer</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Lucas TVS</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Chennai, Tamil Nadu</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>2-4 Yrs</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Multithreading, Debugging, Data Structures, C++14/17</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Today</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-lead-c-developer-lucas-tvs-nk_a18e067e?src=seo_srp&amp;sid=1700000000</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>2026-09-28 18:31:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>nk_b8c2006f</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>C++ Developer</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Wipro</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Chennai (Hybrid)</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>1-3 Yrs</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>OOP, Multithreading, Socket Programming, Linux, Algorithms, STL</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>1 Day Ago</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-c-developer-wipro-nk_b8c2006f?src=seo_srp&amp;sid=1700000000</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>2026-09-28 18:31:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>nk_a8f7257a</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>C++ Developer</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Sify Technologies</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Chennai - All Areas</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>2-5 Yrs</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>C++, Data Structures, Socket Programming, Linux, STL, Debugging, Multithreading</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>3 Days Ago</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-c-developer-sify-technologies-nk_a8f7257a?src=seo_srp&amp;sid=1700000000</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>2026-09-28 18:31:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>nk_fc04519b</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Principal C++ Developer Architect</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>HCLTech</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Chennai (Hybrid)</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>4-8 Yrs</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Multithreading, Linux, C++14/17, OOP, STL</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Just Now</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-principal-c-developer-architect-hcltech-nk_fc04519b?src=seo_srp&amp;sid=1700000000</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>2026-09-28 18:31:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>nk_318c07ba</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>C++ Developer (Backend / Systems)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Lucas TVS</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Chennai / Chennai</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>4-8 Yrs</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Linux, OOP, Data Structures, C++, Algorithms, Socket Programming</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Just Now</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-c-developer-backend-systems-lucas-tvs-nk_318c07ba?src=seo_srp&amp;sid=1700000000</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>2026-09-28 18:31:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>nk_53b8b515</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Software Engineer - C++ Developer</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>HCLTech</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Chennai (Hybrid)</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>2-5 Yrs</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Socket Programming, OOP, STL, Multithreading, Debugging</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Just Now</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-software-engineer-c-developer-hcltech-nk_53b8b515?src=seo_srp&amp;sid=1700000000</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>2026-09-28 18:31:05</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I11"/>
+  <autoFilter ref="A1:I28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add real-time history search, individual delete, and delete all features
</commit_message>
<xml_diff>
--- a/data/naukri_jobs.xlsx
+++ b/data/naukri_jobs.xlsx
@@ -8,19 +8,15 @@
   </bookViews>
   <sheets>
     <sheet name="Master History" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Java Devoper - Chennai" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="PYTHON Devoloper - delhi" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="PYTHON Devoloper - Chennai" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Java Devoper - delhi" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="c++ developer - Chennai" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="PYTHON Devoloper - delhi" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="PYTHON Devoloper - Chennai" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="c++ developer - Chennai" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Master History'!$A$1:$K$69</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Java Devoper - Chennai'!$A$1:$I$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'PYTHON Devoloper - delhi'!$A$1:$I$29</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'PYTHON Devoloper - Chennai'!$A$1:$I$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Java Devoper - delhi'!$A$1:$I$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'c++ developer - Chennai'!$A$1:$I$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Master History'!$A$1:$I$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'PYTHON Devoloper - delhi'!$A$1:$I$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'PYTHON Devoloper - Chennai'!$A$1:$I$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'c++ developer - Chennai'!$A$1:$I$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -451,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K69"/>
+  <dimension ref="A1:I68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -466,272 +462,232 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Search</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>Keyword</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>Location</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Job ID</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>Title</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>Company</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>Experience</t>
-        </is>
-      </c>
-      <c r="H1" s="2" t="inlineStr">
-        <is>
-          <t>Skills</t>
-        </is>
-      </c>
-      <c r="I1" s="2" t="inlineStr">
-        <is>
-          <t>Posted Date</t>
-        </is>
-      </c>
-      <c r="J1" s="2" t="inlineStr">
-        <is>
-          <t>Job URL</t>
-        </is>
-      </c>
-      <c r="K1" s="2" t="inlineStr">
-        <is>
-          <t>Scraped At</t>
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>job_id</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>location</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>experience</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>posted_date</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>job_url</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>scraped_at</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>Java Devoper - Chennai</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>Java Devoper</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>Chennai</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>270826030432</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>Privilega Access management + Azure Devoper</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>Statusneo Technology Consulting</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>7-12 Yrs</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>Identity Access ManagementTerraformPIMIdentity ManagementAzure SecurityPowershellPAMAzure DevOps</t>
-        </is>
-      </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>030226500926</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Frontend devoloper</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Bluphlux</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>3-5 Yrs</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>frontend developmentrestfront endcssuxversion controlui developmentbootstrap</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>3+ weeks ago</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-frontend-devoloper-bluphlux-hyderabad-3-to-5-years-030226500926</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-09-15 21:24:51</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>100924500984</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Software Architect</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Thyssenkrupp Polysius</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Pune</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>5-8 Yrs</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>ProcurementHibernateSoftware designCodingAgileWorkflowHealthcareScrum</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>3+ weeks ago</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-software-architect-thyssenkrupp-polysius-pune-5-to-8-years-100924500984</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-09-15 21:24:51</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>190826037520</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Python Software Developer</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Infosys</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Hybrid - Delhi / NCR, Kolkata, Pune</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2-3 Yrs</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>DjangoPythonFlaskSoftwareSoftware developmentDevelopment</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>2 weeks ago</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>https://www.naukri.com/job-listings-privilega-access-management-azure-devoper-statusneo-technology-consulting-bengaluru-7-to-12-years-270826030432</t>
-        </is>
-      </c>
-      <c r="K2" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-15 21:20:46</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>PYTHON Devoloper - delhi</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>PYTHON Devoloper</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>delhi</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>030226500926</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Frontend devoloper</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Bluphlux</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>3-5 Yrs</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>frontend developmentrestfront endcssuxversion controlui developmentbootstrap</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>3+ weeks ago</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>https://www.naukri.com/job-listings-frontend-devoloper-bluphlux-hyderabad-3-to-5-years-030226500926</t>
-        </is>
-      </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-15 21:24:51</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>PYTHON Devoloper - delhi</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>PYTHON Devoloper</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>delhi</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>100924500984</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>Software Architect</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Thyssenkrupp Polysius</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>5-8 Yrs</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>ProcurementHibernateSoftware designCodingAgileWorkflowHealthcareScrum</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>3+ weeks ago</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>https://www.naukri.com/job-listings-software-architect-thyssenkrupp-polysius-pune-5-to-8-years-100924500984</t>
-        </is>
-      </c>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-15 21:24:51</t>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-python-software-developer-infosys-kolkata-pune-delhi-ncr-2-to-3-years-190826037520</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2026-09-15 21:40:15</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>190826037520</t>
+          <t>020926033318</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Python Software Developer</t>
+          <t>Python Developer</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Infosys</t>
+          <t>EY</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Hybrid - Delhi / NCR, Kolkata, Pune</t>
+          <t>Hybrid - Delhi / NCR, Hyderabad, Pune</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2-3 Yrs</t>
+          <t>3-8 Yrs</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>DjangoPythonFlaskSoftwareSoftware developmentDevelopment</t>
+          <t>Python DeveloperPython DevelopmentPythonDevelopment</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2 weeks ago</t>
+          <t>1 week ago</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-python-software-developer-infosys-kolkata-pune-delhi-ncr-2-to-3-years-190826037520</t>
+          <t>https://www.naukri.com/job-listings-python-developer-ey-hyderabad-pune-delhi-ncr-3-to-8-years-020926033318</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -743,7 +699,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>020926033318</t>
+          <t>150926924122</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -753,44 +709,44 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>EY</t>
+          <t>Soul Ai</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Hybrid - Delhi / NCR, Hyderabad, Pune</t>
+          <t>Delhi / NCR</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>3-8 Yrs</t>
+          <t>4-8 Yrs</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Python DeveloperPython DevelopmentPythonDevelopment</t>
+          <t>PythonpandasdjangoAI modelsnumpyflaskjavascriptArtificial Intelligence</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>1 week ago</t>
+          <t>Few hours ago</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-python-developer-ey-hyderabad-pune-delhi-ncr-3-to-8-years-020926033318</t>
+          <t>https://www.naukri.com/job-listings-python-developer-soul-ai-delhi-ncr-4-to-8-years-150926924122</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-09-15 21:40:15</t>
+          <t>2026-09-15 21:40:16</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>150926924122</t>
+          <t>150926921876</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -805,17 +761,17 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Delhi / NCR</t>
+          <t>New Delhi</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>4-8 Yrs</t>
+          <t>1-3 Yrs</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>PythonpandasdjangoAI modelsnumpyflaskjavascriptArtificial Intelligence</t>
+          <t>PythonSoftware developmentDjangoFastAPIFlaskSoftwareDevelopmentPython Development</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -825,7 +781,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-python-developer-soul-ai-delhi-ncr-4-to-8-years-150926924122</t>
+          <t>https://www.naukri.com/job-listings-python-developer-soul-ai-new-delhi-1-to-3-years-150926921876</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -837,12 +793,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>150926921876</t>
+          <t>150926923243</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Python Developer</t>
+          <t>Python Developer (Mid-Level)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -857,12 +813,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1-3 Yrs</t>
+          <t>2-4 Yrs</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>PythonSoftware developmentDjangoFastAPIFlaskSoftwareDevelopmentPython Development</t>
+          <t>pythoncssnumpyartificial intelligencejquerysqldockerbuild automation</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -872,7 +828,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-python-developer-soul-ai-new-delhi-1-to-3-years-150926921876</t>
+          <t>https://www.naukri.com/job-listings-python-developer-mid-level-soul-ai-new-delhi-2-to-4-years-150926923243</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -884,42 +840,42 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>150926923243</t>
+          <t>120926013305</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Python Developer (Mid-Level)</t>
+          <t>Python Developer</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Soul Ai</t>
+          <t>Infosys</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>New Delhi</t>
+          <t>Hybrid - Delhi / NCR, Hyderabad, Bengaluru</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2-4 Yrs</t>
+          <t>5-8 Yrs</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>pythoncssnumpyartificial intelligencejquerysqldockerbuild automation</t>
+          <t>pythonNumpysqlPandasetlAutomationData EngineeringAPI Development</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Few hours ago</t>
+          <t>3 days ago</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-python-developer-mid-level-soul-ai-new-delhi-2-to-4-years-150926923243</t>
+          <t>https://www.naukri.com/job-listings-python-developer-infosys-hyderabad-bengaluru-delhi-ncr-5-to-8-years-120926013305</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -931,7 +887,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>120926013305</t>
+          <t>080926032481</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -941,69 +897,69 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Infosys</t>
+          <t>Raygain Technologies</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Hybrid - Delhi / NCR, Hyderabad, Bengaluru</t>
+          <t>New Delhi(Safdarjung Enclave)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>5-8 Yrs</t>
+          <t>3-6 Yrs</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>pythonNumpysqlPandasetlAutomationData EngineeringAPI Development</t>
+          <t>Python Web FrameworkPython Frameworkpython languagePython DevelopmentPythonPython TestingPython Data AnalyticsPython Flask</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>3 days ago</t>
+          <t>1 week ago</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-python-developer-infosys-hyderabad-bengaluru-delhi-ncr-5-to-8-years-120926013305</t>
+          <t>https://www.naukri.com/job-listings-python-developer-raygain-technologies-new-delhi-3-to-6-years-080926032481</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-09-15 21:40:16</t>
+          <t>2026-09-15 21:40:49</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>080926032481</t>
+          <t>040926925968</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Python Developer</t>
+          <t>Python Software Developer</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Raygain Technologies</t>
+          <t>Cloudxtreme</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>New Delhi(Safdarjung Enclave)</t>
+          <t>Delhi / NCR, Hyderabad, Bengaluru</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>3-6 Yrs</t>
+          <t>7-12 Yrs</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Python Web FrameworkPython Frameworkpython languagePython DevelopmentPythonPython TestingPython Data AnalyticsPython Flask</t>
+          <t>RestFast APIPython DevelopmentDjangoAPIPythonSoftwareSoftware development</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1013,7 +969,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-python-developer-raygain-technologies-new-delhi-3-to-6-years-080926032481</t>
+          <t>https://www.naukri.com/job-listings-python-software-developer-cloudxtreme-hyderabad-bengaluru-delhi-ncr-7-to-12-years-040926925968</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1025,32 +981,32 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>040926925968</t>
+          <t>040926008818</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Python Software Developer</t>
+          <t>Python Developer</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Cloudxtreme</t>
+          <t>Innovationm</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Delhi / NCR, Hyderabad, Bengaluru</t>
+          <t>Delhi / NCR, Noida, Gurugram</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>7-12 Yrs</t>
+          <t>3-7 Yrs</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>RestFast APIPython DevelopmentDjangoAPIPythonSoftwareSoftware development</t>
+          <t>PythonDjangoPostgresqlPandasNumpyFlaskDevelopmentPython Development</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1060,7 +1016,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-python-software-developer-cloudxtreme-hyderabad-bengaluru-delhi-ncr-7-to-12-years-040926925968</t>
+          <t>https://www.naukri.com/job-listings-python-developer-innovationm-noida-gurugram-delhi-ncr-3-to-7-years-040926008818</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1072,7 +1028,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>040926008818</t>
+          <t>121124502854</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1082,32 +1038,32 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Innovationm</t>
+          <t>Appzlogic</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Delhi / NCR, Noida, Gurugram</t>
+          <t>New Delhi, Kolkata, Mumbai, Hyderabad, Pune, Chennai, Bengaluru</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>3-7 Yrs</t>
+          <t>0-3 Yrs</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>PythonDjangoPostgresqlPandasNumpyFlaskDevelopmentPython Development</t>
+          <t>pythoncsscsoftware testingnatural language processingpython developmentmachine learningartificial intelligence</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>1 week ago</t>
+          <t>3+ weeks ago</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-python-developer-innovationm-noida-gurugram-delhi-ncr-3-to-7-years-040926008818</t>
+          <t>https://www.naukri.com/job-listings-python-developer-appzlogic-mobility-solutions-pvt-ltd-kolkata-mumbai-new-delhi-hyderabad-pune-chennai-bengaluru-0-to-3-years-121124502854</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1119,7 +1075,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>121124502854</t>
+          <t>010926006913</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1129,32 +1085,32 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Appzlogic</t>
+          <t>Tenacious Hr Solution</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>New Delhi, Kolkata, Mumbai, Hyderabad, Pune, Chennai, Bengaluru</t>
+          <t>Delhi / NCR, Bengaluru, Mumbai (All Areas)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>0-3 Yrs</t>
+          <t>2-7 Yrs</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>pythoncsscsoftware testingnatural language processingpython developmentmachine learningartificial intelligence</t>
+          <t>PythonJavaFullstack DevelopmentJavascriptFull StackNode.jsJava FullstackReact.js</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>3+ weeks ago</t>
+          <t>2 weeks ago</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-python-developer-appzlogic-mobility-solutions-pvt-ltd-kolkata-mumbai-new-delhi-hyderabad-pune-chennai-bengaluru-0-to-3-years-121124502854</t>
+          <t>https://www.naukri.com/job-listings-python-developer-tenacious-hr-solution-bengaluru-delhi-ncr-mumbai-all-areas-2-to-7-years-010926006913</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1166,59 +1122,59 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>010926006913</t>
+          <t>040926925419</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Python Developer</t>
+          <t>Python developer</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Tenacious Hr Solution</t>
+          <t>Cloudxtreme</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Delhi / NCR, Bengaluru, Mumbai (All Areas)</t>
+          <t>Delhi / NCR, Kolkata, Bengaluru</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2-7 Yrs</t>
+          <t>5-9 Yrs</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>PythonJavaFullstack DevelopmentJavascriptFull StackNode.jsJava FullstackReact.js</t>
+          <t>GCPFast APIPython DevelopmentMicroservicesPythonDevelopmentAPI</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2 weeks ago</t>
+          <t>1 week ago</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-python-developer-tenacious-hr-solution-bengaluru-delhi-ncr-mumbai-all-areas-2-to-7-years-010926006913</t>
+          <t>https://www.naukri.com/job-listings-python-developer-cloudxtreme-kolkata-bengaluru-delhi-ncr-5-to-9-years-040926925419</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-09-15 21:40:49</t>
+          <t>2026-09-15 21:40:50</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>040926925419</t>
+          <t>040926928118</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Python developer</t>
+          <t>Python Software Developer</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1228,17 +1184,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Delhi / NCR, Kolkata, Bengaluru</t>
+          <t>Hybrid - Delhi / NCR, Bengaluru, Mumbai (All Areas)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>5-9 Yrs</t>
+          <t>4-9 Yrs</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>GCPFast APIPython DevelopmentMicroservicesPythonDevelopmentAPI</t>
+          <t>GolangGrafanaPythonKuberneteskedagpuSoftwareSoftware development</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1248,7 +1204,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-python-developer-cloudxtreme-kolkata-bengaluru-delhi-ncr-5-to-9-years-040926925419</t>
+          <t>https://www.naukri.com/job-listings-python-software-developer-cloudxtreme-bengaluru-delhi-ncr-mumbai-all-areas-4-to-9-years-040926928118</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1260,32 +1216,32 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>040926928118</t>
+          <t>030926010873</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Python Software Developer</t>
+          <t>Python Developer</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Cloudxtreme</t>
+          <t>Statusneo Technology Consulting</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Hybrid - Delhi / NCR, Bengaluru, Mumbai (All Areas)</t>
+          <t>Delhi / NCR, Bengaluru</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>4-9 Yrs</t>
+          <t>5-10 Yrs</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>GolangGrafanaPythonKuberneteskedagpuSoftwareSoftware development</t>
+          <t>DjangoFast ApiPythonFlaskAPIPython DevelopmentDevelopment</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1295,7 +1251,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-python-software-developer-cloudxtreme-bengaluru-delhi-ncr-mumbai-all-areas-4-to-9-years-040926928118</t>
+          <t>https://www.naukri.com/job-listings-python-developer-statusneo-technology-consulting-bengaluru-delhi-ncr-5-to-10-years-030926010873</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1307,42 +1263,42 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>030926010873</t>
+          <t>010926022053</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Python Developer</t>
+          <t>Python Software Developer</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Statusneo Technology Consulting</t>
+          <t>EY</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Delhi / NCR, Bengaluru</t>
+          <t>Delhi / NCR, Hyderabad, Bengaluru</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>5-10 Yrs</t>
+          <t>4-12 Yrs</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>DjangoFast ApiPythonFlaskAPIPython DevelopmentDevelopment</t>
+          <t>Large Language ModelDjangoFast APIAWSPythonArtificial IntelligenceRetrieval Augmented GenerationFlask</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>1 week ago</t>
+          <t>2 weeks ago</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-python-developer-statusneo-technology-consulting-bengaluru-delhi-ncr-5-to-10-years-030926010873</t>
+          <t>https://www.naukri.com/job-listings-python-software-developer-ey-hyderabad-bengaluru-delhi-ncr-4-to-12-years-010926022053</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1354,32 +1310,32 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>010926022053</t>
+          <t>310826014429</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Python Software Developer</t>
+          <t>Python / AI Developer</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>EY</t>
+          <t>Ommify Technologies</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Delhi / NCR, Hyderabad, Bengaluru</t>
+          <t>New Delhi(Netaji Subhash Place)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>4-12 Yrs</t>
+          <t>1-3 Yrs</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Large Language ModelDjangoFast APIAWSPythonArtificial IntelligenceRetrieval Augmented GenerationFlask</t>
+          <t>API Design and DevelopmentPythonNextjsArtificial IntelligenceDesign developmentDevelopmentDesignDevelopment</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1389,54 +1345,54 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-python-software-developer-ey-hyderabad-bengaluru-delhi-ncr-4-to-12-years-010926022053</t>
+          <t>https://www.naukri.com/job-listings-python-ai-developer-ommify-technologies-new-delhi-1-to-3-years-310826014429</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-09-15 21:40:50</t>
+          <t>2026-09-15 21:40:57</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>310826014429</t>
+          <t>090926033497</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Python / AI Developer</t>
+          <t>Software Developer - Java &amp; Python</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Ommify Technologies</t>
+          <t>MNC</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>New Delhi(Netaji Subhash Place)</t>
+          <t>New Delhi, Gurugram, Delhi / NCR</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1-3 Yrs</t>
+          <t>4-9 Yrs</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>API Design and DevelopmentPythonNextjsArtificial IntelligenceDesign developmentDevelopmentDesignDevelopment</t>
+          <t>JavaJava FullstackJavascriptPython DevelopmentPythonPython FrameworkCi/CdJavascript Frameworks</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2 weeks ago</t>
+          <t>6 days ago</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-python-ai-developer-ommify-technologies-new-delhi-1-to-3-years-310826014429</t>
+          <t>https://www.naukri.com/job-listings-software-developer-java-python-hr-hai-new-delhi-gurugram-delhi-ncr-4-to-9-years-090926033497</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1448,42 +1404,42 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>090926033497</t>
+          <t>190826923056</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Software Developer - Java &amp; Python</t>
+          <t>Python Developer</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>MNC</t>
+          <t>Clouwood Studio</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>New Delhi, Gurugram, Delhi / NCR</t>
+          <t>Delhi / NCR, Hyderabad, Chennai</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>4-9 Yrs</t>
+          <t>2-5 Yrs</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>JavaJava FullstackJavascriptPython DevelopmentPythonPython FrameworkCi/CdJavascript Frameworks</t>
+          <t>python developeremerging technologiespythonsoftware developmentit servicesprogramming languagecommunication and interpersonal skillsprogramming</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>6 days ago</t>
+          <t>3 weeks ago</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-software-developer-java-python-hr-hai-new-delhi-gurugram-delhi-ncr-4-to-9-years-090926033497</t>
+          <t>https://www.naukri.com/job-listings-python-developer-clouwood-studio-hyderabad-chennai-delhi-ncr-2-to-5-years-190826923056</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1495,32 +1451,32 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>190826923056</t>
+          <t>240826004591</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Python Developer</t>
+          <t>Gen AI Python Developer - S</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Clouwood Studio</t>
+          <t>Tata Consultancy Services</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Delhi / NCR, Hyderabad, Chennai</t>
+          <t>Delhi / NCR, Chennai, Bengaluru</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2-5 Yrs</t>
+          <t>4-8 Yrs</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>python developeremerging technologiespythonsoftware developmentit servicesprogramming languagecommunication and interpersonal skillsprogramming</t>
+          <t>generative aiPythonData ManagementMachine LearningSQLArtificial IntelligenceManagementData</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1530,7 +1486,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-python-developer-clouwood-studio-hyderabad-chennai-delhi-ncr-2-to-5-years-190826923056</t>
+          <t>https://www.naukri.com/job-listings-gen-ai-python-developer-s-tata-consultancy-services-chennai-bengaluru-delhi-ncr-4-to-8-years-240826004591</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1542,42 +1498,42 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>240826004591</t>
+          <t>260620500907</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Gen AI Python Developer - S</t>
+          <t>Python Developer</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Tata Consultancy Services</t>
+          <t>Mind Digital Group</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Delhi / NCR, Chennai, Bengaluru</t>
+          <t>New Delhi</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>4-8 Yrs</t>
+          <t>2-7 Yrs</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>generative aiPythonData ManagementMachine LearningSQLArtificial IntelligenceManagementData</t>
+          <t>UnixAutomationLinuxSolarisShell scriptingJavascriptPHPData structures</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>3 weeks ago</t>
+          <t>3+ weeks ago</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-gen-ai-python-developer-s-tata-consultancy-services-chennai-bengaluru-delhi-ncr-4-to-8-years-240826004591</t>
+          <t>https://www.naukri.com/job-listings-python-developer-mind-digital-group-delhi-2-to-7-years-260620500907</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1589,32 +1545,32 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>260620500907</t>
+          <t>200226504783</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Python Developer</t>
+          <t>Python Developer | Infosys</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mind Digital Group</t>
+          <t>Logic Planet</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>New Delhi</t>
+          <t>New Delhi, Kolkata, Mumbai, Hyderabad, Pune, Chennai, Bengaluru</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2-7 Yrs</t>
+          <t>7-10 Yrs</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>UnixAutomationLinuxSolarisShell scriptingJavascriptPHPData structures</t>
+          <t>restpythonrestfulversion controldata processingcloud platformspython developercaching</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1624,24 +1580,24 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-python-developer-mind-digital-group-delhi-2-to-7-years-260620500907</t>
+          <t>https://www.naukri.com/job-listings-python-developer-infosys-logicplanet-it-services-kolkata-mumbai-new-delhi-hyderabad-pune-chennai-bengaluru-7-to-10-years-200226504783</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-09-15 21:40:57</t>
+          <t>2026-09-15 21:40:58</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>200226504783</t>
+          <t>200226504901</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Python Developer | Infosys</t>
+          <t>Python Developer</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1656,12 +1612,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>7-10 Yrs</t>
+          <t>6-10 Yrs</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>restpythonrestfulversion controldata processingcloud platformspython developercaching</t>
+          <t>pythoncssrestfulsoftware developmentpython developerjavascriptmicroservicesdatabase design</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1671,7 +1627,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-python-developer-infosys-logicplanet-it-services-kolkata-mumbai-new-delhi-hyderabad-pune-chennai-bengaluru-7-to-10-years-200226504783</t>
+          <t>https://www.naukri.com/job-listings-python-developer-logicplanet-it-services-kolkata-mumbai-new-delhi-hyderabad-pune-chennai-bengaluru-6-to-10-years-200226504901</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1683,42 +1639,42 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>200226504901</t>
+          <t>310826017377</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Python Developer</t>
+          <t>Python / AI Developer</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Logic Planet</t>
+          <t>National e-Governance Division</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>New Delhi, Kolkata, Mumbai, Hyderabad, Pune, Chennai, Bengaluru</t>
+          <t>Delhi / NCR</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>6-10 Yrs</t>
+          <t>3-5 Yrs</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>pythoncssrestfulsoftware developmentpython developerjavascriptmicroservicesdatabase design</t>
+          <t>Artificial IntelligencePythonSoftware EngineeringMachine LearningDeep LearningIntelligenceEngineeringSoftware</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>3+ weeks ago</t>
+          <t>2 weeks ago</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-python-developer-logicplanet-it-services-kolkata-mumbai-new-delhi-hyderabad-pune-chennai-bengaluru-6-to-10-years-200226504901</t>
+          <t>https://www.naukri.com/job-listings-python-ai-developer-national-e-governance-division-delhi-ncr-3-to-5-years-310826017377</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1730,42 +1686,42 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>310826017377</t>
+          <t>090925500511</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Python / AI Developer</t>
+          <t>Python Developer</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>National e-Governance Division</t>
+          <t>Photon</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Delhi / NCR</t>
+          <t>New Delhi, Kolkata, Mumbai, Hyderabad, Pune, Chennai, Bengaluru</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>3-5 Yrs</t>
+          <t>3-8 Yrs</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Artificial IntelligencePythonSoftware EngineeringMachine LearningDeep LearningIntelligenceEngineeringSoftware</t>
+          <t>JAXGCPCloud ServicesProgrammingTransformersAWSPythonProgram</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2 weeks ago</t>
+          <t>3+ weeks ago</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-python-ai-developer-national-e-governance-division-delhi-ncr-3-to-5-years-310826017377</t>
+          <t>https://www.naukri.com/job-listings-python-developer-photon-infotech-p-ltd-kolkata-mumbai-new-delhi-hyderabad-pune-chennai-bengaluru-3-to-8-years-090925500511</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1777,7 +1733,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>090925500511</t>
+          <t>190825500726</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1787,7 +1743,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Photon</t>
+          <t>Aark Global</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1797,12 +1753,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>3-8 Yrs</t>
+          <t>5-10 Yrs</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>JAXGCPCloud ServicesProgrammingTransformersAWSPythonProgram</t>
+          <t>C++AutomationDb2CodingScrumOracleTroubleshootingInformation technology</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1812,7 +1768,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-python-developer-photon-infotech-p-ltd-kolkata-mumbai-new-delhi-hyderabad-pune-chennai-bengaluru-3-to-8-years-090925500511</t>
+          <t>https://www.naukri.com/job-listings-python-developer-aark-global-inc-kolkata-mumbai-new-delhi-hyderabad-pune-chennai-bengaluru-5-to-10-years-190825500726</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1824,22 +1780,22 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>190825500726</t>
+          <t>190826011177</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Python Developer</t>
+          <t>Agentic AI and Python Developer</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Aark Global</t>
+          <t>Sapient (publicissapient)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>New Delhi, Kolkata, Mumbai, Hyderabad, Pune, Chennai, Bengaluru</t>
+          <t>Delhi / NCR, Gurugram, Bengaluru</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1849,17 +1805,17 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>C++AutomationDb2CodingScrumOracleTroubleshootingInformation technology</t>
+          <t>Agentic AiPython DevelopmentPythonDevelopmentArtificial Intelligence</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>3+ weeks ago</t>
+          <t>3 weeks ago</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-python-developer-aark-global-inc-kolkata-mumbai-new-delhi-hyderabad-pune-chennai-bengaluru-5-to-10-years-190825500726</t>
+          <t>https://www.naukri.com/job-listings-agentic-ai-and-python-developer-sapient-publicissapient-gurugram-bengaluru-delhi-ncr-5-to-10-years-190826011177</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1871,64 +1827,64 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>190826011177</t>
+          <t>300826004292</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Agentic AI and Python Developer</t>
+          <t>Python GenAI Developer</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Sapient (publicissapient)</t>
+          <t>Tata Consultancy Services</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Delhi / NCR, Gurugram, Bengaluru</t>
+          <t>Chennai</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>5-10 Yrs</t>
+          <t>4-9 Yrs</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Agentic AiPython DevelopmentPythonDevelopmentArtificial Intelligence</t>
+          <t>GenAIRAG FrameworkPythonLLMFrameworkDevelopment</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>3 weeks ago</t>
+          <t>2 weeks ago</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-agentic-ai-and-python-developer-sapient-publicissapient-gurugram-bengaluru-delhi-ncr-5-to-10-years-190826011177</t>
+          <t>https://www.naukri.com/job-listings-python-genai-developer-tata-consultancy-services-chennai-4-to-9-years-300826004292</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-09-15 21:40:58</t>
+          <t>2026-09-15 21:44:15</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>300826004292</t>
+          <t>260826500429</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Python GenAI Developer</t>
+          <t>Python Developer</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Tata Consultancy Services</t>
+          <t>UST</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1938,12 +1894,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>4-9 Yrs</t>
+          <t>5-7 Yrs</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>GenAIRAG FrameworkPythonLLMFrameworkDevelopment</t>
+          <t>api developmentdebugbusiness requirementscloud platformsagile developmentbug fixingdockercloud</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1953,7 +1909,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-python-genai-developer-tata-consultancy-services-chennai-4-to-9-years-300826004292</t>
+          <t>https://www.naukri.com/job-listings-python-developer-ust-chennai-5-to-7-years-260826500429</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -1965,17 +1921,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>260826500429</t>
+          <t>110926020162</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Python Developer</t>
+          <t>Walk-in || Python Software Developer</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>UST</t>
+          <t>Meythoma International</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1985,44 +1941,44 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>5-7 Yrs</t>
+          <t>12 Sep - 19 Sep</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>api developmentdebugbusiness requirementscloud platformsagile developmentbug fixingdockercloud</t>
+          <t>PythonDjangoSQLSoftwareSoftware developmentDevelopment</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2 weeks ago</t>
+          <t>4 days ago</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-python-developer-ust-chennai-5-to-7-years-260826500429</t>
+          <t>https://www.naukri.com/job-listings-python-software-developer-meythoma-international-chennai-0-to-3-years-110926020162</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-09-15 21:44:15</t>
+          <t>2026-09-15 21:44:16</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>110926020162</t>
+          <t>080926501298</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Walk-in || Python Software Developer</t>
+          <t>Python Developer</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Meythoma International</t>
+          <t>Tridots Tech</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2032,22 +1988,22 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>12 Sep - 19 Sep</t>
+          <t>0-2 Yrs</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>PythonDjangoSQLSoftwareSoftware developmentDevelopment</t>
+          <t>csspythondebugagile developmentbootstrappython developerweb applicationsjavascript</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>4 days ago</t>
+          <t>1 week ago</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-python-software-developer-meythoma-international-chennai-0-to-3-years-110926020162</t>
+          <t>https://www.naukri.com/job-listings-python-developer-tridots-tech-private-limited-chennai-0-to-2-years-080926501298</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2059,17 +2015,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>080926501298</t>
+          <t>140926004200</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Python Developer</t>
+          <t>Walk-in || Python Software Developer</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Tridots Tech</t>
+          <t>Tata Consultancy Services</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2079,22 +2035,22 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>0-2 Yrs</t>
+          <t>19 Sep</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>csspythondebugagile developmentbootstrappython developerweb applicationsjavascript</t>
+          <t>Djangopython developerNumpyScipyPandasSoftwarePythonSoftware development</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>1 week ago</t>
+          <t>1 day ago</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-python-developer-tridots-tech-private-limited-chennai-0-to-2-years-080926501298</t>
+          <t>https://www.naukri.com/job-listings-python-software-developer-tata-consultancy-services-chennai-4-to-9-years-140926004200</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2106,17 +2062,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>140926004200</t>
+          <t>100926917183</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Walk-in || Python Software Developer</t>
+          <t>Python Senior Software Developer</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Tata Consultancy Services</t>
+          <t>Kaspon</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -2126,22 +2082,22 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>19 Sep</t>
+          <t>4-5 Yrs</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Djangopython developerNumpyScipyPandasSoftwarePythonSoftware development</t>
+          <t>Angular 8PythonBDDMVVMTrelloHTMLAngular 8 &amp; AboveRESTAPI</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>1 day ago</t>
+          <t>5 days ago</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-python-software-developer-tata-consultancy-services-chennai-4-to-9-years-140926004200</t>
+          <t>https://www.naukri.com/job-listings-python-senior-software-developer-kaspontech-techworks-chennai-4-to-5-years-100926917183</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2153,17 +2109,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>100926917183</t>
+          <t>100926933981</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Python Senior Software Developer</t>
+          <t>Python Developer</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Kaspon</t>
+          <t>Infosys</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2173,12 +2129,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>4-5 Yrs</t>
+          <t>3-5 Yrs</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Angular 8PythonBDDMVVMTrelloHTMLAngular 8 &amp; AboveRESTAPI</t>
+          <t>PythonCssPostgresqlArtificial IntelligenceData StructuresNatural Language ProcessingHtmlMachine Learning</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2188,29 +2144,29 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-python-senior-software-developer-kaspontech-techworks-chennai-4-to-5-years-100926917183</t>
+          <t>https://www.naukri.com/job-listings-python-developer-infosys-limited-chennai-3-to-5-years-100926933981</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-09-15 21:44:16</t>
+          <t>2026-09-15 21:44:23</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>100926933981</t>
+          <t>090926008196</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Python Developer</t>
+          <t>Walk-in || Python Software Developer</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Infosys</t>
+          <t>Tata Consultancy Services</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2220,22 +2176,22 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>3-5 Yrs</t>
+          <t>19 Sep</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>PythonCssPostgresqlArtificial IntelligenceData StructuresNatural Language ProcessingHtmlMachine Learning</t>
+          <t>NumpyPythonPython DevelopmentSoftwareSoftware developmentDevelopment</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>5 days ago</t>
+          <t>6 days ago</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-python-developer-infosys-limited-chennai-3-to-5-years-100926933981</t>
+          <t>https://www.naukri.com/job-listings-python-software-developer-tata-consultancy-services-chennai-4-to-9-years-090926008196</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2247,12 +2203,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>090926008196</t>
+          <t>100926017827</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Walk-in || Python Software Developer</t>
+          <t>Python Software Developer</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2267,22 +2223,22 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>19 Sep</t>
+          <t>4-9 Yrs</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>NumpyPythonPython DevelopmentSoftwareSoftware developmentDevelopment</t>
+          <t>Python DevelopmentDockerNumpySoftwarePythonSoftware developmentDevelopment</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>6 days ago</t>
+          <t>5 days ago</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-python-software-developer-tata-consultancy-services-chennai-4-to-9-years-090926008196</t>
+          <t>https://www.naukri.com/job-listings-python-software-developer-tata-consultancy-services-chennai-4-to-9-years-100926017827</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2294,12 +2250,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>100926017827</t>
+          <t>100926018290</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Python Software Developer</t>
+          <t>Walk-in || Python Software Developer</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2314,12 +2270,12 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>4-9 Yrs</t>
+          <t>19 Sep</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Python DevelopmentDockerNumpySoftwarePythonSoftware developmentDevelopment</t>
+          <t>PythonRESTful APIRest Web APIDjangoRestful WebFlaskAPIRest Web</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2329,19 +2285,19 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-python-software-developer-tata-consultancy-services-chennai-4-to-9-years-100926017827</t>
+          <t>https://www.naukri.com/job-listings-python-software-developer-tata-consultancy-services-chennai-4-to-9-years-100926018290</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-09-15 21:44:23</t>
+          <t>2026-09-15 21:44:24</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>100926018290</t>
+          <t>110926002993</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2366,17 +2322,17 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>PythonRESTful APIRest Web APIDjangoRestful WebFlaskAPIRest Web</t>
+          <t>PythonAzure CloudGCPDjangoPandasCi/CdPython DevelopmentRest API Development</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>5 days ago</t>
+          <t>4 days ago</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-python-software-developer-tata-consultancy-services-chennai-4-to-9-years-100926018290</t>
+          <t>https://www.naukri.com/job-listings-python-software-developer-tata-consultancy-services-chennai-4-to-9-years-110926002993</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -2388,12 +2344,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>110926002993</t>
+          <t>110926013972</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Walk-in || Python Software Developer</t>
+          <t>Walk-in || Python Developer</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2413,7 +2369,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>PythonAzure CloudGCPDjangoPandasCi/CdPython DevelopmentRest API Development</t>
+          <t>Python FrameworkPython DevelopmentMachine LearningPythonFrameworkDevelopmentMachine</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2423,7 +2379,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-python-software-developer-tata-consultancy-services-chennai-4-to-9-years-110926002993</t>
+          <t>https://www.naukri.com/job-listings-python-developer-tata-consultancy-services-chennai-4-to-9-years-110926013972</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2435,17 +2391,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>110926013972</t>
+          <t>150926933774</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Walk-in || Python Developer</t>
+          <t>C# Developer</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Tata Consultancy Services</t>
+          <t>Soul Ai</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2455,44 +2411,44 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>19 Sep</t>
+          <t>2-4 Yrs</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Python FrameworkPython DevelopmentMachine LearningPythonFrameworkDevelopmentMachine</t>
+          <t>c#asp.net.netweb apimvcvisualforcec++dml</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>4 days ago</t>
+          <t>2 days ago</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-python-developer-tata-consultancy-services-chennai-4-to-9-years-110926013972</t>
+          <t>https://www.naukri.com/job-listings-c-developer-soul-ai-chennai-2-to-4-years-150926933774</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>2026-09-15 21:44:24</t>
+          <t>2026-09-18 14:48:52</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>150926933774</t>
+          <t>170926501465</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>C# Developer</t>
+          <t>Embedded C++ Developer</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Soul Ai</t>
+          <t>ITC Infotech</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -2502,22 +2458,22 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2-4 Yrs</t>
+          <t>3-7 Yrs</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>c#asp.net.netweb apimvcvisualforcec++dml</t>
+          <t>RTOSMechatronicsCMINLinuxWindowsFirmwareOpen source</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>2 days ago</t>
+          <t>1 day ago</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-c-developer-soul-ai-chennai-2-to-4-years-150926933774</t>
+          <t>https://www.naukri.com/job-listings-embedded-c-developer-itc-infotech-india-ltd-chennai-3-to-7-years-170926501465</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -2529,17 +2485,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>170926501465</t>
+          <t>160926939901</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Embedded C++ Developer</t>
+          <t>Typescript and C++ Developer</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>ITC Infotech</t>
+          <t>FIS</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -2549,12 +2505,12 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>3-7 Yrs</t>
+          <t>6-11 Yrs</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>RTOSMechatronicsCMINLinuxWindowsFirmwareOpen source</t>
+          <t>Api GatewayApplication SoftwareAzureFinancial ServicesFintechCloud ServicesGithubBanking</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2564,7 +2520,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-embedded-c-developer-itc-infotech-india-ltd-chennai-3-to-7-years-170926501465</t>
+          <t>https://www.naukri.com/job-listings-typescript-and-c-developer-fis-global-business-solutions-india-pvt-ltd-chennai-6-to-11-years-160926939901</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2576,17 +2532,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>160926939901</t>
+          <t>070926918874</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Typescript and C++ Developer</t>
+          <t>BSW Developer(SoC)</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>FIS</t>
+          <t>ZF</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -2596,44 +2552,44 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>6-11 Yrs</t>
+          <t>4-7 Yrs</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Api GatewayApplication SoftwareAzureFinancial ServicesFintechCloud ServicesGithubBanking</t>
+          <t>ArchitectureRtosProcessorPrototypeSocSoftware ArchitectureAutosarProgramming</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>1 day ago</t>
+          <t>1 week ago</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-typescript-and-c-developer-fis-global-business-solutions-india-pvt-ltd-chennai-6-to-11-years-160926939901</t>
+          <t>https://www.naukri.com/job-listings-bsw-developer-soc-zf-india-private-limited-chennai-4-to-7-years-070926918874</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>2026-09-18 14:48:52</t>
+          <t>2026-09-18 14:48:53</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>070926918874</t>
+          <t>100926031501</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>BSW Developer(SoC)</t>
+          <t>Embedded C++ Developer</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>ZF</t>
+          <t>Expleo</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2643,12 +2599,12 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>4-7 Yrs</t>
+          <t>5-10 Yrs</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>ArchitectureRtosProcessorPrototypeSocSoftware ArchitectureAutosarProgramming</t>
+          <t>Embedded C++LeadAutomotiveEmbedded developmentC++DevelopmentEmbedded systemsEmbedded Firmware Development</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2658,7 +2614,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-bsw-developer-soc-zf-india-private-limited-chennai-4-to-7-years-070926918874</t>
+          <t>https://www.naukri.com/job-listings-embedded-c-developer-expleo-chennai-5-to-10-years-100926031501</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -2670,17 +2626,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>100926031501</t>
+          <t>150926934283</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Embedded C++ Developer</t>
+          <t>C++ Developer</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Expleo</t>
+          <t>Soul Ai</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2690,22 +2646,22 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>5-10 Yrs</t>
+          <t>2-4 Yrs</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Embedded C++LeadAutomotiveEmbedded developmentC++DevelopmentEmbedded systemsEmbedded Firmware Development</t>
+          <t>c#c++asp.net.netmvcvisualforcedmlsoftware development</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>1 week ago</t>
+          <t>2 days ago</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-embedded-c-developer-expleo-chennai-5-to-10-years-100926031501</t>
+          <t>https://www.naukri.com/job-listings-c-developer-soul-ai-chennai-2-to-4-years-150926934283</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -2717,17 +2673,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>150926934283</t>
+          <t>110926909175</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>C++ Developer</t>
+          <t>C++ Developer (IST/Switch)</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Soul Ai</t>
+          <t>FIS</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2737,22 +2693,22 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>2-4 Yrs</t>
+          <t>5-10 Yrs</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>c#c++asp.net.netmvcvisualforcedmlsoftware development</t>
+          <t>AgileEnterprise ApplicationsFinancial ServicesArchitectureFintechDesign PatternsConcurrentData Structures</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>2 days ago</t>
+          <t>1 week ago</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-c-developer-soul-ai-chennai-2-to-4-years-150926934283</t>
+          <t>https://www.naukri.com/job-listings-c-developer-ist-switch-fis-global-business-solutions-india-pvt-ltd-chennai-5-to-10-years-110926909175</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -2764,12 +2720,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>110926909175</t>
+          <t>110926003784</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>C++ Developer (IST/Switch)</t>
+          <t>C++ Developer</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2784,12 +2740,12 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>5-10 Yrs</t>
+          <t>4-9 Yrs</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>AgileEnterprise ApplicationsFinancial ServicesArchitectureFintechDesign PatternsConcurrentData Structures</t>
+          <t>C++IST SwitchPaymentsDevelopment</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2799,7 +2755,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-c-developer-ist-switch-fis-global-business-solutions-india-pvt-ltd-chennai-5-to-10-years-110926909175</t>
+          <t>https://www.naukri.com/job-listings-c-developer-fis-chennai-4-to-9-years-110926003784</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -2811,12 +2767,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>110926003784</t>
+          <t>310826916472</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>C++ Developer</t>
+          <t>C++ Developer with IST Switch</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2831,22 +2787,22 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>4-9 Yrs</t>
+          <t>5-10 Yrs</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>C++IST SwitchPaymentsDevelopment</t>
+          <t>bankingoraclefintechretailjavac++ developmentpospayment domain</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>1 week ago</t>
+          <t>2 weeks ago</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-c-developer-fis-chennai-4-to-9-years-110926003784</t>
+          <t>https://www.naukri.com/job-listings-c-developer-with-ist-switch-fis-global-business-solutions-india-pvt-ltd-chennai-5-to-10-years-310826916472</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -2858,17 +2814,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>310826916472</t>
+          <t>240826001555</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>C++ Developer with IST Switch</t>
+          <t>C++ Developer</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>FIS</t>
+          <t>Danfoss</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -2878,106 +2834,106 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>5-10 Yrs</t>
+          <t>5-14 Yrs</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>bankingoraclefintechretailjavac++ developmentpospayment domain</t>
+          <t>C++ Object Oriented ProgrammingMultithreadingDesign DevelopmentLinuxMultithread ProgrammingDesign PatternsNetwork ProgrammingSTL</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>2 weeks ago</t>
+          <t>3 weeks ago</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-c-developer-with-ist-switch-fis-global-business-solutions-india-pvt-ltd-chennai-5-to-10-years-310826916472</t>
+          <t>https://www.naukri.com/job-listings-c-developer-danfoss-chennai-5-to-14-years-240826001555</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>2026-09-18 14:48:53</t>
+          <t>2026-09-18 14:48:54</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>240826001555</t>
+          <t>nk_e916fe98</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>C++ Developer</t>
+          <t>C++ Developer Module Lead</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Danfoss</t>
+          <t>Ramco Systems</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Chennai</t>
+          <t>Chennai - All Areas</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>5-14 Yrs</t>
+          <t>2-4 Yrs</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>C++ Object Oriented ProgrammingMultithreadingDesign DevelopmentLinuxMultithread ProgrammingDesign PatternsNetwork ProgrammingSTL</t>
+          <t>C++14/17, Algorithms, OOP, Socket Programming, Data Structures</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>3 weeks ago</t>
+          <t>3 Days Ago</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-c-developer-danfoss-chennai-5-to-14-years-240826001555</t>
+          <t>https://www.naukri.com/job-listings-c-developer-module-lead-ramco-systems-nk_e916fe98?src=seo_srp&amp;sid=1700000000</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>2026-09-18 14:48:54</t>
+          <t>2026-09-28 18:31:05</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>nk_e916fe98</t>
+          <t>nk_eef6e622</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>C++ Developer Module Lead</t>
+          <t>C++ Developer Application Developer</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Ramco Systems</t>
+          <t>HCLTech</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Chennai - All Areas</t>
+          <t>Chennai</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>2-4 Yrs</t>
+          <t>5-10 Yrs</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>C++14/17, Algorithms, OOP, Socket Programming, Data Structures</t>
+          <t>Data Structures, STL, OOP, Debugging, Socket Programming</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -2987,7 +2943,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-c-developer-module-lead-ramco-systems-nk_e916fe98?src=seo_srp&amp;sid=1700000000</t>
+          <t>https://www.naukri.com/job-listings-c-developer-application-developer-hcltech-nk_eef6e622?src=seo_srp&amp;sid=1700000000</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -2999,42 +2955,42 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>nk_eef6e622</t>
+          <t>nk_e6472a94</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>C++ Developer Application Developer</t>
+          <t>C++ Developer Module Lead</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>HCLTech</t>
+          <t>Wipro</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Chennai</t>
+          <t>Chennai / Chennai</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>5-10 Yrs</t>
+          <t>4-8 Yrs</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Data Structures, STL, OOP, Debugging, Socket Programming</t>
+          <t>Linux, Data Structures, Algorithms, C++, Socket Programming, Debugging, OOP</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>3 Days Ago</t>
+          <t>Today</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-c-developer-application-developer-hcltech-nk_eef6e622?src=seo_srp&amp;sid=1700000000</t>
+          <t>https://www.naukri.com/job-listings-c-developer-module-lead-wipro-nk_e6472a94?src=seo_srp&amp;sid=1700000000</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -3046,42 +3002,42 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>nk_e6472a94</t>
+          <t>nk_94f42425</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>C++ Developer Module Lead</t>
+          <t>Senior C++ Developer</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Wipro</t>
+          <t>Ford Global Technology</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Chennai / Chennai</t>
+          <t>Chennai, Tamil Nadu</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>4-8 Yrs</t>
+          <t>0-2 Yrs</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Linux, Data Structures, Algorithms, C++, Socket Programming, Debugging, OOP</t>
+          <t>Socket Programming, STL, C++14/17, C++, Data Structures, Algorithms, Multithreading</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Today</t>
+          <t>1 Day Ago</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-c-developer-module-lead-wipro-nk_e6472a94?src=seo_srp&amp;sid=1700000000</t>
+          <t>https://www.naukri.com/job-listings-senior-c-developer-ford-global-technology-nk_94f42425?src=seo_srp&amp;sid=1700000000</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3093,42 +3049,42 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>nk_94f42425</t>
+          <t>nk_2c2c41b0</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Senior C++ Developer</t>
+          <t>Junior C++ Developer</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Ford Global Technology</t>
+          <t>Ramco Systems</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Chennai, Tamil Nadu</t>
+          <t>Chennai</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>0-2 Yrs</t>
+          <t>1-3 Yrs</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Socket Programming, STL, C++14/17, C++, Data Structures, Algorithms, Multithreading</t>
+          <t>STL, OOP, C++, Linux, Debugging</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>1 Day Ago</t>
+          <t>Just Now</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-senior-c-developer-ford-global-technology-nk_94f42425?src=seo_srp&amp;sid=1700000000</t>
+          <t>https://www.naukri.com/job-listings-junior-c-developer-ramco-systems-nk_2c2c41b0?src=seo_srp&amp;sid=1700000000</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -3140,17 +3096,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>nk_2c2c41b0</t>
+          <t>nk_9bc8de7c</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Junior C++ Developer</t>
+          <t>Principal C++ Developer Architect</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Ramco Systems</t>
+          <t>Zoho Corporation</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -3160,22 +3116,22 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>1-3 Yrs</t>
+          <t>4-8 Yrs</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>STL, OOP, C++, Linux, Debugging</t>
+          <t>Algorithms, Debugging, C++, STL, OOP, Data Structures, Socket Programming</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Just Now</t>
+          <t>Today</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-junior-c-developer-ramco-systems-nk_2c2c41b0?src=seo_srp&amp;sid=1700000000</t>
+          <t>https://www.naukri.com/job-listings-principal-c-developer-architect-zoho-corporation-nk_9bc8de7c?src=seo_srp&amp;sid=1700000000</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -3187,42 +3143,42 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>nk_9bc8de7c</t>
+          <t>nk_7590cad9</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Principal C++ Developer Architect</t>
+          <t>C++ Developer (Backend / Systems)</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Zoho Corporation</t>
+          <t>Infosys Chennai</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Chennai</t>
+          <t>Chennai - All Areas</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>4-8 Yrs</t>
+          <t>1-3 Yrs</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Algorithms, Debugging, C++, STL, OOP, Data Structures, Socket Programming</t>
+          <t>OOP, Socket Programming, C++, Multithreading, Algorithms, STL, C++14/17</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Today</t>
+          <t>Just Now</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-principal-c-developer-architect-zoho-corporation-nk_9bc8de7c?src=seo_srp&amp;sid=1700000000</t>
+          <t>https://www.naukri.com/job-listings-c-developer-backend-systems-infosys-chennai-nk_7590cad9?src=seo_srp&amp;sid=1700000000</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -3234,42 +3190,42 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>nk_7590cad9</t>
+          <t>nk_5801a5b5</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>C++ Developer (Backend / Systems)</t>
+          <t>C++ Developer Module Lead</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Infosys Chennai</t>
+          <t>Sify Technologies</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Chennai - All Areas</t>
+          <t>Chennai / Chennai</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>1-3 Yrs</t>
+          <t>2-5 Yrs</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>OOP, Socket Programming, C++, Multithreading, Algorithms, STL, C++14/17</t>
+          <t>OOP, Linux, Multithreading, Algorithms</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Just Now</t>
+          <t>2 Days Ago</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-c-developer-backend-systems-infosys-chennai-nk_7590cad9?src=seo_srp&amp;sid=1700000000</t>
+          <t>https://www.naukri.com/job-listings-c-developer-module-lead-sify-technologies-nk_5801a5b5?src=seo_srp&amp;sid=1700000000</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -3281,42 +3237,42 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>nk_5801a5b5</t>
+          <t>nk_5b46595c</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>C++ Developer Module Lead</t>
+          <t>C++ Developer (Backend / Systems)</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Sify Technologies</t>
+          <t>Amazon Chennai</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Chennai / Chennai</t>
+          <t>Chennai, Tamil Nadu</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>2-5 Yrs</t>
+          <t>0-2 Yrs</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>OOP, Linux, Multithreading, Algorithms</t>
+          <t>Debugging, OOP, Socket Programming, Multithreading, Linux</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>2 Days Ago</t>
+          <t>1 Day Ago</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-c-developer-module-lead-sify-technologies-nk_5801a5b5?src=seo_srp&amp;sid=1700000000</t>
+          <t>https://www.naukri.com/job-listings-c-developer-backend-systems-amazon-chennai-nk_5b46595c?src=seo_srp&amp;sid=1700000000</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -3328,17 +3284,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>nk_5b46595c</t>
+          <t>nk_add002bc</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>C++ Developer (Backend / Systems)</t>
+          <t>Associate C++ Developer</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Amazon Chennai</t>
+          <t>HCLTech</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -3353,17 +3309,17 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Debugging, OOP, Socket Programming, Multithreading, Linux</t>
+          <t>Socket Programming, OOP, Multithreading, Algorithms</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>1 Day Ago</t>
+          <t>Today</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-c-developer-backend-systems-amazon-chennai-nk_5b46595c?src=seo_srp&amp;sid=1700000000</t>
+          <t>https://www.naukri.com/job-listings-associate-c-developer-hcltech-nk_add002bc?src=seo_srp&amp;sid=1700000000</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -3375,7 +3331,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>nk_add002bc</t>
+          <t>nk_5d7a5b82</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3385,32 +3341,32 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>HCLTech</t>
+          <t>Wipro</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Chennai, Tamil Nadu</t>
+          <t>Chennai (Hybrid)</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>0-2 Yrs</t>
+          <t>5-10 Yrs</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Socket Programming, OOP, Multithreading, Algorithms</t>
+          <t>Linux, Debugging, Multithreading, OOP</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Today</t>
+          <t>Few Hours Ago</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-associate-c-developer-hcltech-nk_add002bc?src=seo_srp&amp;sid=1700000000</t>
+          <t>https://www.naukri.com/job-listings-associate-c-developer-wipro-nk_5d7a5b82?src=seo_srp&amp;sid=1700000000</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -3422,42 +3378,42 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>nk_5d7a5b82</t>
+          <t>nk_a18e067e</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Associate C++ Developer</t>
+          <t>Lead C++ Developer</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Wipro</t>
+          <t>Lucas TVS</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Chennai (Hybrid)</t>
+          <t>Chennai, Tamil Nadu</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>5-10 Yrs</t>
+          <t>2-4 Yrs</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Linux, Debugging, Multithreading, OOP</t>
+          <t>Multithreading, Debugging, Data Structures, C++14/17</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Few Hours Ago</t>
+          <t>Today</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-associate-c-developer-wipro-nk_5d7a5b82?src=seo_srp&amp;sid=1700000000</t>
+          <t>https://www.naukri.com/job-listings-lead-c-developer-lucas-tvs-nk_a18e067e?src=seo_srp&amp;sid=1700000000</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -3469,42 +3425,42 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>nk_a18e067e</t>
+          <t>nk_b8c2006f</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Lead C++ Developer</t>
+          <t>C++ Developer</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Lucas TVS</t>
+          <t>Wipro</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Chennai, Tamil Nadu</t>
+          <t>Chennai (Hybrid)</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>2-4 Yrs</t>
+          <t>1-3 Yrs</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Multithreading, Debugging, Data Structures, C++14/17</t>
+          <t>OOP, Multithreading, Socket Programming, Linux, Algorithms, STL</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Today</t>
+          <t>1 Day Ago</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-lead-c-developer-lucas-tvs-nk_a18e067e?src=seo_srp&amp;sid=1700000000</t>
+          <t>https://www.naukri.com/job-listings-c-developer-wipro-nk_b8c2006f?src=seo_srp&amp;sid=1700000000</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -3516,7 +3472,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>nk_b8c2006f</t>
+          <t>nk_a8f7257a</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3526,32 +3482,32 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Wipro</t>
+          <t>Sify Technologies</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Chennai (Hybrid)</t>
+          <t>Chennai - All Areas</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>1-3 Yrs</t>
+          <t>2-5 Yrs</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>OOP, Multithreading, Socket Programming, Linux, Algorithms, STL</t>
+          <t>C++, Data Structures, Socket Programming, Linux, STL, Debugging, Multithreading</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>1 Day Ago</t>
+          <t>3 Days Ago</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-c-developer-wipro-nk_b8c2006f?src=seo_srp&amp;sid=1700000000</t>
+          <t>https://www.naukri.com/job-listings-c-developer-sify-technologies-nk_a8f7257a?src=seo_srp&amp;sid=1700000000</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -3563,42 +3519,42 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>nk_a8f7257a</t>
+          <t>nk_fc04519b</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>C++ Developer</t>
+          <t>Principal C++ Developer Architect</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Sify Technologies</t>
+          <t>HCLTech</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Chennai - All Areas</t>
+          <t>Chennai (Hybrid)</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>2-5 Yrs</t>
+          <t>4-8 Yrs</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>C++, Data Structures, Socket Programming, Linux, STL, Debugging, Multithreading</t>
+          <t>Multithreading, Linux, C++14/17, OOP, STL</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>3 Days Ago</t>
+          <t>Just Now</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-c-developer-sify-technologies-nk_a8f7257a?src=seo_srp&amp;sid=1700000000</t>
+          <t>https://www.naukri.com/job-listings-principal-c-developer-architect-hcltech-nk_fc04519b?src=seo_srp&amp;sid=1700000000</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -3610,22 +3566,22 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>nk_fc04519b</t>
+          <t>nk_318c07ba</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Principal C++ Developer Architect</t>
+          <t>C++ Developer (Backend / Systems)</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>HCLTech</t>
+          <t>Lucas TVS</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Chennai (Hybrid)</t>
+          <t>Chennai / Chennai</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -3635,7 +3591,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Multithreading, Linux, C++14/17, OOP, STL</t>
+          <t>Linux, OOP, Data Structures, C++, Algorithms, Socket Programming</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -3645,7 +3601,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-principal-c-developer-architect-hcltech-nk_fc04519b?src=seo_srp&amp;sid=1700000000</t>
+          <t>https://www.naukri.com/job-listings-c-developer-backend-systems-lucas-tvs-nk_318c07ba?src=seo_srp&amp;sid=1700000000</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -3657,32 +3613,32 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>nk_318c07ba</t>
+          <t>nk_53b8b515</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>C++ Developer (Backend / Systems)</t>
+          <t>Software Engineer - C++ Developer</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Lucas TVS</t>
+          <t>HCLTech</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Chennai / Chennai</t>
+          <t>Chennai (Hybrid)</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>4-8 Yrs</t>
+          <t>2-5 Yrs</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Linux, OOP, Data Structures, C++, Algorithms, Socket Programming</t>
+          <t>Socket Programming, OOP, STL, Multithreading, Debugging</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -3692,179 +3648,12 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/job-listings-c-developer-backend-systems-lucas-tvs-nk_318c07ba?src=seo_srp&amp;sid=1700000000</t>
+          <t>https://www.naukri.com/job-listings-software-engineer-c-developer-hcltech-nk_53b8b515?src=seo_srp&amp;sid=1700000000</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
           <t>2026-09-28 18:31:05</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>nk_53b8b515</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>Software Engineer - C++ Developer</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>HCLTech</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>Chennai (Hybrid)</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>2-5 Yrs</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>Socket Programming, OOP, STL, Multithreading, Debugging</t>
-        </is>
-      </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>Just Now</t>
-        </is>
-      </c>
-      <c r="H69" t="inlineStr">
-        <is>
-          <t>https://www.naukri.com/job-listings-software-engineer-c-developer-hcltech-nk_53b8b515?src=seo_srp&amp;sid=1700000000</t>
-        </is>
-      </c>
-      <c r="I69" t="inlineStr">
-        <is>
-          <t>2026-09-28 18:31:05</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:K69"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="65" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="80" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>job_id</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>company</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>location</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>experience</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>skills</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>posted_date</t>
-        </is>
-      </c>
-      <c r="H1" s="2" t="inlineStr">
-        <is>
-          <t>job_url</t>
-        </is>
-      </c>
-      <c r="I1" s="2" t="inlineStr">
-        <is>
-          <t>scraped_at</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>270826030432</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>Privilega Access management + Azure Devoper</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>Statusneo Technology Consulting</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>Bengaluru</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>7-12 Yrs</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>Identity Access ManagementTerraformPIMIdentity ManagementAzure SecurityPowershellPAMAzure DevOps</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>2 weeks ago</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>https://www.naukri.com/job-listings-privilega-access-management-azure-devoper-statusneo-technology-consulting-bengaluru-7-to-12-years-270826030432</t>
-        </is>
-      </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-15 21:20:46</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3663,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5263,7 +5052,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5900,80 +5689,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="65" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="85" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>job_id</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>company</t>
-        </is>
-      </c>
-      <c r="D1" s="4" t="inlineStr">
-        <is>
-          <t>location</t>
-        </is>
-      </c>
-      <c r="E1" s="4" t="inlineStr">
-        <is>
-          <t>experience</t>
-        </is>
-      </c>
-      <c r="F1" s="4" t="inlineStr">
-        <is>
-          <t>skills</t>
-        </is>
-      </c>
-      <c r="G1" s="4" t="inlineStr">
-        <is>
-          <t>posted_date</t>
-        </is>
-      </c>
-      <c r="H1" s="4" t="inlineStr">
-        <is>
-          <t>job_url</t>
-        </is>
-      </c>
-      <c r="I1" s="4" t="inlineStr">
-        <is>
-          <t>scraped_at</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:I1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>